<commit_message>
stabilize ecommerce manual loop and update QA snapshot
</commit_message>
<xml_diff>
--- a/docs/qa/system-use-cases-report.xlsx
+++ b/docs/qa/system-use-cases-report.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Contrato vivo'!A1:M137</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Hallazgos'!A1:I2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Hallazgos'!A1:I4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Guia manual'!A1:K137</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Ecommerce'!A1:L55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Admin'!A1:L43</definedName>
@@ -465,7 +465,7 @@
         <v>Notas</v>
       </c>
       <c r="B5" t="str">
-        <v>Contrato vivo del sistema: VERIFICADA = corrida/paso validado; DEFINIDA = existe cobertura alineada pero no rerun en este informe; PENDIENTE = no existe prueba automatizada suficiente todavía. La hoja Contrato vivo normaliza tipo, inputs, outputs, sistemas involucrados, dependencias, estado y trazabilidad. La hoja Hallazgos queda como registro de errores con clasificación obligatoria. Para este proceso se excluye Chat Platform y se trabaja sobre ecommerce, backend, analytics e integraciones auxiliares. Los bloques de auto-respuesta, wording registry, hybrid intent y grounding quedan fuera del gate de esta entrega manual-only.</v>
+        <v>Contrato vivo del sistema: VERIFICADA = corrida/paso validado; DEFINIDA = existe cobertura alineada pero no rerun en este informe; PENDIENTE = no existe prueba automatizada suficiente todavía. La hoja Contrato vivo normaliza tipo, inputs, outputs, sistemas involucrados, dependencias, estado y trazabilidad. La hoja Hallazgos queda como registro de errores con clasificación obligatoria. Para este proceso se excluye Chat Platform y cualquier chat automatizado con IA; el foco manual queda en Meta, Mail y Webchat. Snapshot de manuales 2026-05-03: ecommerce crítico de checkout quedó verde y el bloque manual de canales quedó en 18/18; mantener como punto de partida para la siguiente iteración.</v>
       </c>
     </row>
     <row r="7">
@@ -6319,16 +6319,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I4"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="46.83203125" customWidth="1"/>
+    <col min="5" max="5" width="52.83203125" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" customWidth="1"/>
     <col min="7" max="7" width="37.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="52.83203125" customWidth="1"/>
     <col min="9" max="9" width="52.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6363,37 +6363,95 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>QA-ECOM-VITEST-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>deuda técnica</v>
+      </c>
+      <c r="C2" t="str">
+        <v>frontend</v>
+      </c>
+      <c r="D2" t="str">
+        <v>helpers storefront/SEO y render de contenido CMS</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Ejecutar `cd ecommerce &amp;&amp; npx vitest run` con la configuración actual del repo.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>media</v>
+      </c>
+      <c r="G2" t="str">
+        <v>open</v>
+      </c>
+      <c r="H2" t="str">
+        <v>ecommerce/src/lib/page-metadata.spec.ts; ecommerce/src/lib/seo/robots.spec.ts; ecommerce/src/lib/seo/sitemap.spec.ts; ecommerce/src/lib/seo/public-pricing.spec.ts; ecommerce/src/lib/seo/structured-data.spec.ts; ecommerce/src/lib/analytics/eventSchema.spec.ts; ecommerce/src/components/cms/rich-text.spec.ts</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Las suites fallan antes de llegar a las aserciones con un error de lectura sobre `config`; hay que normalizar el setup de vitest o corregir la dependencia que asume un entorno distinto.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>QA-ECOM-ADMIN-AI-001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>bug funcional</v>
+      </c>
+      <c r="C3" t="str">
+        <v>frontend</v>
+      </c>
+      <c r="D3" t="str">
+        <v>admin AI settings / knowledge management</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Ejecutar `cd ecommerce &amp;&amp; npx playwright test --workers=1 e2e/admin-ai-settings.spec.ts`.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>alta</v>
+      </c>
+      <c r="G3" t="str">
+        <v>open</v>
+      </c>
+      <c r="H3" t="str">
+        <v>ecommerce/e2e/admin-ai-settings.spec.ts</v>
+      </c>
+      <c r="I3" t="str">
+        <v>La corrida quedó fallando en navegación a runtime settings, creación/reindexado de knowledge y pantallas de documentos; requiere validación funcional antes de cerrar manuales.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
         <v/>
       </c>
-      <c r="B2" t="str">
+      <c r="B4" t="str">
         <v>bug funcional | inconsistencia entre servicios | desalineación con documento | gap funcional | deuda técnica</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C4" t="str">
         <v/>
       </c>
-      <c r="D2" t="str">
+      <c r="D4" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
+      <c r="E4" t="str">
         <v/>
       </c>
-      <c r="F2" t="str">
+      <c r="F4" t="str">
         <v>crítica | media | baja</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G4" t="str">
         <v>open | in_progress | fixed | validated</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="I4" t="str">
         <v>Registrar evidencia, impacto cruzado y decisión de documentación. Completar una fila por hallazgo real.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>